<commit_message>
updated report directory path and modified branch references in CI configuration
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/data.xlsx
+++ b/src/test/java/TestData/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>Username</t>
   </si>
@@ -27,6 +27,10 @@
   <si>
     <t xml:space="preserve">12345678!
 </t>
+  </si>
+  <si>
+    <t>" bugmagnet@gmail.com 
+"</t>
   </si>
 </sst>
 </file>
@@ -329,7 +333,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.13"/>
+    <col customWidth="1" min="1" max="1" width="26.25"/>
     <col customWidth="1" min="2" max="2" width="12.88"/>
     <col customWidth="1" min="3" max="26" width="8.88"/>
   </cols>
@@ -351,8 +355,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4"/>

</xml_diff>